<commit_message>
update max attempts for course test
</commit_message>
<xml_diff>
--- a/public/templates/format_course_test.xlsx
+++ b/public/templates/format_course_test.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/muchammadalifzaidan/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F0589BF-4373-5A40-87E2-22A195816EEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAAB1546-0B0E-8A46-A187-BF6EE8B0225C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="23260" windowHeight="12460" xr2:uid="{E30444BF-1D59-4066-BE44-2A4D90506F0C}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="17">
   <si>
     <t>title</t>
   </si>
@@ -82,6 +82,9 @@
   </si>
   <si>
     <t>question_bank_name</t>
+  </si>
+  <si>
+    <t>max_attempts</t>
   </si>
 </sst>
 </file>
@@ -475,7 +478,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65CC1420-A9E4-4CB7-B8CB-64A2A3DACE1E}">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="23.5" customWidth="1"/>
@@ -485,9 +488,11 @@
     <col min="6" max="6" width="15.6640625" customWidth="1"/>
     <col min="7" max="7" width="22.5" customWidth="1"/>
     <col min="8" max="8" width="18.33203125" customWidth="1"/>
+    <col min="9" max="9" width="14.83203125" customWidth="1"/>
+    <col min="10" max="10" width="13.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -515,8 +520,11 @@
       <c r="I1" s="6" t="s">
         <v>7</v>
       </c>
+      <c r="J1" s="6" t="s">
+        <v>16</v>
+      </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -544,8 +552,11 @@
       <c r="I2" t="b">
         <v>1</v>
       </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -573,8 +584,11 @@
       <c r="I3" t="b">
         <v>1</v>
       </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B4" s="1"/>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>

</xml_diff>

<commit_message>
feat: add show_correct_answers configuration to course tests and update result visibility logic in UI
</commit_message>
<xml_diff>
--- a/public/templates/format_course_test.xlsx
+++ b/public/templates/format_course_test.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/muchammadalifzaidan/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/muchammadalifzaidan/Development/Project/brevetlearning/public/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAAB1546-0B0E-8A46-A187-BF6EE8B0225C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B5C60EE-41E0-2A42-89D5-BF836DA5DD20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="23260" windowHeight="12460" xr2:uid="{E30444BF-1D59-4066-BE44-2A4D90506F0C}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="18">
   <si>
     <t>title</t>
   </si>
@@ -85,6 +85,9 @@
   </si>
   <si>
     <t>max_attempts</t>
+  </si>
+  <si>
+    <t>show_correct_answers</t>
   </si>
 </sst>
 </file>
@@ -478,7 +481,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65CC1420-A9E4-4CB7-B8CB-64A2A3DACE1E}">
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="23.5" customWidth="1"/>
@@ -490,9 +493,10 @@
     <col min="8" max="8" width="18.33203125" customWidth="1"/>
     <col min="9" max="9" width="14.83203125" customWidth="1"/>
     <col min="10" max="10" width="13.5" customWidth="1"/>
+    <col min="11" max="11" width="19.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -523,8 +527,11 @@
       <c r="J1" s="6" t="s">
         <v>16</v>
       </c>
+      <c r="K1" s="6" t="s">
+        <v>17</v>
+      </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -555,8 +562,11 @@
       <c r="J2">
         <v>0</v>
       </c>
+      <c r="K2" t="b">
+        <v>1</v>
+      </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -587,8 +597,11 @@
       <c r="J3">
         <v>0</v>
       </c>
+      <c r="K3" t="b">
+        <v>1</v>
+      </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B4" s="1"/>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>

</xml_diff>